<commit_message>
feat(gui): combobox de dataset + separacao maior v2
- Seletor de dataset alterado de radio buttons para Label + Combobox
  em ambas as abas (layout: 'Dataset:  [dropdown]')
- Margem de separacao do iris_data_02 aumentada de 0.08 para 1.5
  no espaco discriminante (aprox. 1 cm fisico em petalas); 72 amostras
  ajustadas gerando gap visual claro entre versicolor e virginica
- theme.py: estilo TCombobox adicionado ao aplicar_tema
</commit_message>
<xml_diff>
--- a/data/iris_data_02.xlsx
+++ b/data/iris_data_02.xlsx
@@ -1374,10 +1374,10 @@
         <v>3.2</v>
       </c>
       <c r="C51" t="n">
-        <v>4.7</v>
+        <v>4.077326155578938</v>
       </c>
       <c r="D51" t="n">
-        <v>1.4</v>
+        <v>1.062638009988589</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>3.2</v>
       </c>
       <c r="C52" t="n">
-        <v>4.5</v>
+        <v>3.990055678231101</v>
       </c>
       <c r="D52" t="n">
-        <v>1.5</v>
+        <v>1.223714376750597</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1412,10 +1412,10 @@
         <v>3.1</v>
       </c>
       <c r="C53" t="n">
-        <v>4.9</v>
+        <v>4.080827348578034</v>
       </c>
       <c r="D53" t="n">
-        <v>1.5</v>
+        <v>1.056175808053115</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1431,10 +1431,10 @@
         <v>2.3</v>
       </c>
       <c r="C54" t="n">
-        <v>4</v>
+        <v>3.960360374646176</v>
       </c>
       <c r="D54" t="n">
-        <v>1.3</v>
+        <v>1.278523422795916</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1450,10 +1450,10 @@
         <v>2.8</v>
       </c>
       <c r="C55" t="n">
-        <v>4.6</v>
+        <v>4.012748595817834</v>
       </c>
       <c r="D55" t="n">
-        <v>1.5</v>
+        <v>1.181829734576227</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1469,10 +1469,10 @@
         <v>2.8</v>
       </c>
       <c r="C56" t="n">
-        <v>4.5</v>
+        <v>4.073824962579842</v>
       </c>
       <c r="D56" t="n">
-        <v>1.3</v>
+        <v>1.069100211924063</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1488,10 +1488,10 @@
         <v>3.3</v>
       </c>
       <c r="C57" t="n">
-        <v>4.7</v>
+        <v>3.993556871230197</v>
       </c>
       <c r="D57" t="n">
-        <v>1.6</v>
+        <v>1.217252174815122</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1526,10 +1526,10 @@
         <v>2.9</v>
       </c>
       <c r="C59" t="n">
-        <v>4.6</v>
+        <v>4.096517880166575</v>
       </c>
       <c r="D59" t="n">
-        <v>1.3</v>
+        <v>1.027215569749693</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1545,10 +1545,10 @@
         <v>2.7</v>
       </c>
       <c r="C60" t="n">
-        <v>3.9</v>
+        <v>3.895782814885072</v>
       </c>
       <c r="D60" t="n">
-        <v>1.4</v>
+        <v>1.397715147383553</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1583,10 +1583,10 @@
         <v>3</v>
       </c>
       <c r="C62" t="n">
-        <v>4.2</v>
+        <v>3.921976925470902</v>
       </c>
       <c r="D62" t="n">
-        <v>1.5</v>
+        <v>1.349368303273708</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         <v>2.9</v>
       </c>
       <c r="C64" t="n">
-        <v>4.7</v>
+        <v>4.077326155578938</v>
       </c>
       <c r="D64" t="n">
-        <v>1.4</v>
+        <v>1.062638009988589</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1659,10 +1659,10 @@
         <v>3.1</v>
       </c>
       <c r="C66" t="n">
-        <v>4.4</v>
+        <v>4.009247402818739</v>
       </c>
       <c r="D66" t="n">
-        <v>1.4</v>
+        <v>1.1882919365117</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1678,10 +1678,10 @@
         <v>3</v>
       </c>
       <c r="C67" t="n">
-        <v>4.5</v>
+        <v>3.990055678231101</v>
       </c>
       <c r="D67" t="n">
-        <v>1.5</v>
+        <v>1.223714376750597</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1716,10 +1716,10 @@
         <v>2.2</v>
       </c>
       <c r="C69" t="n">
-        <v>4.5</v>
+        <v>3.990055678231101</v>
       </c>
       <c r="D69" t="n">
-        <v>1.5</v>
+        <v>1.223714376750597</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1754,10 +1754,10 @@
         <v>3.2</v>
       </c>
       <c r="C71" t="n">
-        <v>4.782140388576848</v>
+        <v>3.932480504468189</v>
       </c>
       <c r="D71" t="n">
-        <v>1.790323739941017</v>
+        <v>1.329981697467285</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -1773,10 +1773,10 @@
         <v>2.8</v>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>3.960360374646176</v>
       </c>
       <c r="D72" t="n">
-        <v>1.3</v>
+        <v>1.278523422795916</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -1792,10 +1792,10 @@
         <v>2.5</v>
       </c>
       <c r="C73" t="n">
-        <v>4.9</v>
+        <v>4.080827348578034</v>
       </c>
       <c r="D73" t="n">
-        <v>1.5</v>
+        <v>1.056175808053115</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -1811,10 +1811,10 @@
         <v>2.8</v>
       </c>
       <c r="C74" t="n">
-        <v>4.7</v>
+        <v>4.16109543992768</v>
       </c>
       <c r="D74" t="n">
-        <v>1.2</v>
+        <v>0.9080238451620553</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -1830,10 +1830,10 @@
         <v>2.9</v>
       </c>
       <c r="C75" t="n">
-        <v>4.3</v>
+        <v>4.028439127406376</v>
       </c>
       <c r="D75" t="n">
-        <v>1.3</v>
+        <v>1.152869496272804</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -1849,10 +1849,10 @@
         <v>3</v>
       </c>
       <c r="C76" t="n">
-        <v>4.4</v>
+        <v>4.009247402818739</v>
       </c>
       <c r="D76" t="n">
-        <v>1.4</v>
+        <v>1.1882919365117</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1868,10 +1868,10 @@
         <v>2.8</v>
       </c>
       <c r="C77" t="n">
-        <v>4.8</v>
+        <v>4.100019073165671</v>
       </c>
       <c r="D77" t="n">
-        <v>1.4</v>
+        <v>1.020753367814218</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -1887,10 +1887,10 @@
         <v>3</v>
       </c>
       <c r="C78" t="n">
-        <v>4.869410865924685</v>
+        <v>4.019750981816026</v>
       </c>
       <c r="D78" t="n">
-        <v>1.629247373179009</v>
+        <v>1.168905330705277</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1906,10 +1906,10 @@
         <v>2.9</v>
       </c>
       <c r="C79" t="n">
-        <v>4.5</v>
+        <v>3.990055678231101</v>
       </c>
       <c r="D79" t="n">
-        <v>1.5</v>
+        <v>1.223714376750597</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2001,10 +2001,10 @@
         <v>2.7</v>
       </c>
       <c r="C84" t="n">
-        <v>4.933988425685788</v>
+        <v>4.084328541577129</v>
       </c>
       <c r="D84" t="n">
-        <v>1.510055648591372</v>
+        <v>1.049713606117641</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2020,10 +2020,10 @@
         <v>3</v>
       </c>
       <c r="C85" t="n">
-        <v>4.5</v>
+        <v>3.990055678231101</v>
       </c>
       <c r="D85" t="n">
-        <v>1.5</v>
+        <v>1.223714376750597</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2039,10 +2039,10 @@
         <v>3.4</v>
       </c>
       <c r="C86" t="n">
-        <v>4.5</v>
+        <v>3.94817103605673</v>
       </c>
       <c r="D86" t="n">
-        <v>1.6</v>
+        <v>1.301021459163863</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2058,10 +2058,10 @@
         <v>3.1</v>
       </c>
       <c r="C87" t="n">
-        <v>4.7</v>
+        <v>4.035441513404567</v>
       </c>
       <c r="D87" t="n">
-        <v>1.5</v>
+        <v>1.139945092401856</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2077,10 +2077,10 @@
         <v>2.3</v>
       </c>
       <c r="C88" t="n">
-        <v>4.4</v>
+        <v>4.051132044993109</v>
       </c>
       <c r="D88" t="n">
-        <v>1.3</v>
+        <v>1.110984854098434</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2096,10 +2096,10 @@
         <v>3</v>
       </c>
       <c r="C89" t="n">
-        <v>4.1</v>
+        <v>3.983053292232909</v>
       </c>
       <c r="D89" t="n">
-        <v>1.3</v>
+        <v>1.236638780621545</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2115,10 +2115,10 @@
         <v>2.5</v>
       </c>
       <c r="C90" t="n">
-        <v>4</v>
+        <v>3.960360374646176</v>
       </c>
       <c r="D90" t="n">
-        <v>1.3</v>
+        <v>1.278523422795916</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2134,10 +2134,10 @@
         <v>2.6</v>
       </c>
       <c r="C91" t="n">
-        <v>4.4</v>
+        <v>4.09301668716748</v>
       </c>
       <c r="D91" t="n">
-        <v>1.2</v>
+        <v>1.033677771685167</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2153,10 +2153,10 @@
         <v>3</v>
       </c>
       <c r="C92" t="n">
-        <v>4.6</v>
+        <v>4.054633237992205</v>
       </c>
       <c r="D92" t="n">
-        <v>1.4</v>
+        <v>1.10452265216296</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2210,10 +2210,10 @@
         <v>2.7</v>
       </c>
       <c r="C95" t="n">
-        <v>4.2</v>
+        <v>4.005746209819643</v>
       </c>
       <c r="D95" t="n">
-        <v>1.3</v>
+        <v>1.194754138447175</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2229,10 +2229,10 @@
         <v>3</v>
       </c>
       <c r="C96" t="n">
-        <v>4.2</v>
+        <v>4.047630851994013</v>
       </c>
       <c r="D96" t="n">
-        <v>1.2</v>
+        <v>1.117447056033908</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>2.9</v>
       </c>
       <c r="C97" t="n">
-        <v>4.2</v>
+        <v>4.005746209819643</v>
       </c>
       <c r="D97" t="n">
-        <v>1.3</v>
+        <v>1.194754138447175</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2267,10 +2267,10 @@
         <v>2.9</v>
       </c>
       <c r="C98" t="n">
-        <v>4.3</v>
+        <v>4.028439127406376</v>
       </c>
       <c r="D98" t="n">
-        <v>1.3</v>
+        <v>1.152869496272804</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2305,10 +2305,10 @@
         <v>2.8</v>
       </c>
       <c r="C100" t="n">
-        <v>4.1</v>
+        <v>3.983053292232909</v>
       </c>
       <c r="D100" t="n">
-        <v>1.3</v>
+        <v>1.236638780621545</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2343,10 +2343,10 @@
         <v>2.7</v>
       </c>
       <c r="C102" t="n">
-        <v>5.1</v>
+        <v>5.753730708241326</v>
       </c>
       <c r="D102" t="n">
-        <v>1.9</v>
+        <v>2.254188464217437</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2381,10 +2381,10 @@
         <v>2.9</v>
       </c>
       <c r="C104" t="n">
-        <v>5.6</v>
+        <v>5.909079938349363</v>
       </c>
       <c r="D104" t="n">
-        <v>1.8</v>
+        <v>1.967458170932317</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2438,10 +2438,10 @@
         <v>2.5</v>
       </c>
       <c r="C107" t="n">
-        <v>4.851682602961009</v>
+        <v>5.701342487069668</v>
       </c>
       <c r="D107" t="n">
-        <v>1.890540109963395</v>
+        <v>2.350882152437126</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2476,10 +2476,10 @@
         <v>2.5</v>
       </c>
       <c r="C109" t="n">
-        <v>5.8</v>
+        <v>5.954465773522829</v>
       </c>
       <c r="D109" t="n">
-        <v>1.8</v>
+        <v>1.883688886583576</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2514,10 +2514,10 @@
         <v>3.2</v>
       </c>
       <c r="C111" t="n">
-        <v>5.1</v>
+        <v>5.711846066066955</v>
       </c>
       <c r="D111" t="n">
-        <v>2</v>
+        <v>2.331495546630703</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2533,10 +2533,10 @@
         <v>2.7</v>
       </c>
       <c r="C112" t="n">
-        <v>5.3</v>
+        <v>5.799116543414793</v>
       </c>
       <c r="D112" t="n">
-        <v>1.9</v>
+        <v>2.170419179868695</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2552,10 +2552,10 @@
         <v>3</v>
       </c>
       <c r="C113" t="n">
-        <v>5.5</v>
+        <v>5.760733094239518</v>
       </c>
       <c r="D113" t="n">
-        <v>2.1</v>
+        <v>2.241264060346488</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2571,10 +2571,10 @@
         <v>2.5</v>
       </c>
       <c r="C114" t="n">
-        <v>5</v>
+        <v>5.689153148480223</v>
       </c>
       <c r="D114" t="n">
-        <v>2</v>
+        <v>2.373380188805074</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2590,10 +2590,10 @@
         <v>2.8</v>
       </c>
       <c r="C115" t="n">
-        <v>5.1</v>
+        <v>5.544307497369473</v>
       </c>
       <c r="D115" t="n">
-        <v>2.4</v>
+        <v>2.64072387628377</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2609,10 +2609,10 @@
         <v>3.2</v>
       </c>
       <c r="C116" t="n">
-        <v>5.3</v>
+        <v>5.631577974717311</v>
       </c>
       <c r="D116" t="n">
-        <v>2.3</v>
+        <v>2.479647509521762</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -2628,10 +2628,10 @@
         <v>3</v>
       </c>
       <c r="C117" t="n">
-        <v>5.5</v>
+        <v>5.88638702076263</v>
       </c>
       <c r="D117" t="n">
-        <v>1.8</v>
+        <v>2.009342813106688</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -2685,10 +2685,10 @@
         <v>2.2</v>
       </c>
       <c r="C120" t="n">
-        <v>5.048916475243416</v>
+        <v>5.898576359352075</v>
       </c>
       <c r="D120" t="n">
-        <v>1.526502734265009</v>
+        <v>1.98684477673874</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -2704,10 +2704,10 @@
         <v>3.2</v>
       </c>
       <c r="C121" t="n">
-        <v>5.7</v>
+        <v>5.722349645064243</v>
       </c>
       <c r="D121" t="n">
-        <v>2.3</v>
+        <v>2.31210894082428</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -2723,10 +2723,10 @@
         <v>2.8</v>
       </c>
       <c r="C122" t="n">
-        <v>4.9</v>
+        <v>5.666460230893489</v>
       </c>
       <c r="D122" t="n">
-        <v>2</v>
+        <v>2.415264830979444</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -2761,10 +2761,10 @@
         <v>2.7</v>
       </c>
       <c r="C124" t="n">
-        <v>4.900569631133572</v>
+        <v>5.75022951524223</v>
       </c>
       <c r="D124" t="n">
-        <v>1.80030862367918</v>
+        <v>2.260650666152911</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2780,10 +2780,10 @@
         <v>3.3</v>
       </c>
       <c r="C125" t="n">
-        <v>5.7</v>
+        <v>5.806118929412984</v>
       </c>
       <c r="D125" t="n">
-        <v>2.1</v>
+        <v>2.157494775997747</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2818,10 +2818,10 @@
         <v>2.8</v>
       </c>
       <c r="C127" t="n">
-        <v>4.877876713546838</v>
+        <v>5.727536597655497</v>
       </c>
       <c r="D127" t="n">
-        <v>1.84219326585355</v>
+        <v>2.302535308327282</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -2837,10 +2837,10 @@
         <v>3</v>
       </c>
       <c r="C128" t="n">
-        <v>4.900569631133572</v>
+        <v>5.75022951524223</v>
       </c>
       <c r="D128" t="n">
-        <v>1.80030862367918</v>
+        <v>2.260650666152911</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2856,10 +2856,10 @@
         <v>2.8</v>
       </c>
       <c r="C129" t="n">
-        <v>5.6</v>
+        <v>5.783426011826251</v>
       </c>
       <c r="D129" t="n">
-        <v>2.1</v>
+        <v>2.199379418172118</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -2875,10 +2875,10 @@
         <v>3</v>
       </c>
       <c r="C130" t="n">
-        <v>5.8</v>
+        <v>6.038235057871571</v>
       </c>
       <c r="D130" t="n">
-        <v>1.6</v>
+        <v>1.729074721757043</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -2932,10 +2932,10 @@
         <v>2.8</v>
       </c>
       <c r="C133" t="n">
-        <v>5.6</v>
+        <v>5.74154136965188</v>
       </c>
       <c r="D133" t="n">
-        <v>2.2</v>
+        <v>2.276686500585384</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -2951,10 +2951,10 @@
         <v>2.8</v>
       </c>
       <c r="C134" t="n">
-        <v>5.1</v>
+        <v>5.921269276938808</v>
       </c>
       <c r="D134" t="n">
-        <v>1.5</v>
+        <v>1.94496013456437</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2970,10 +2970,10 @@
         <v>2.6</v>
       </c>
       <c r="C135" t="n">
-        <v>5.6</v>
+        <v>6.076618507046845</v>
       </c>
       <c r="D135" t="n">
-        <v>1.4</v>
+        <v>1.65822984127925</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3008,10 +3008,10 @@
         <v>3.4</v>
       </c>
       <c r="C137" t="n">
-        <v>5.6</v>
+        <v>5.657772085303139</v>
       </c>
       <c r="D137" t="n">
-        <v>2.4</v>
+        <v>2.431300665411918</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3027,10 +3027,10 @@
         <v>3.1</v>
       </c>
       <c r="C138" t="n">
-        <v>5.5</v>
+        <v>5.88638702076263</v>
       </c>
       <c r="D138" t="n">
-        <v>1.8</v>
+        <v>2.009342813106688</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3046,10 +3046,10 @@
         <v>3</v>
       </c>
       <c r="C139" t="n">
-        <v>4.877876713546838</v>
+        <v>5.727536597655497</v>
       </c>
       <c r="D139" t="n">
-        <v>1.84219326585355</v>
+        <v>2.302535308327282</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3065,10 +3065,10 @@
         <v>3.1</v>
       </c>
       <c r="C140" t="n">
-        <v>5.4</v>
+        <v>5.738040176652785</v>
       </c>
       <c r="D140" t="n">
-        <v>2.1</v>
+        <v>2.283148702520858</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3084,10 +3084,10 @@
         <v>3.1</v>
       </c>
       <c r="C141" t="n">
-        <v>5.6</v>
+        <v>5.657772085303139</v>
       </c>
       <c r="D141" t="n">
-        <v>2.4</v>
+        <v>2.431300665411918</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3103,10 +3103,10 @@
         <v>3.1</v>
       </c>
       <c r="C142" t="n">
-        <v>5.1</v>
+        <v>5.586192139543845</v>
       </c>
       <c r="D142" t="n">
-        <v>2.3</v>
+        <v>2.563416793870504</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3122,10 +3122,10 @@
         <v>2.7</v>
       </c>
       <c r="C143" t="n">
-        <v>5.1</v>
+        <v>5.753730708241326</v>
       </c>
       <c r="D143" t="n">
-        <v>1.9</v>
+        <v>2.254188464217437</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3179,10 +3179,10 @@
         <v>3</v>
       </c>
       <c r="C146" t="n">
-        <v>5.2</v>
+        <v>5.608885057130578</v>
       </c>
       <c r="D146" t="n">
-        <v>2.3</v>
+        <v>2.521532151696133</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3198,10 +3198,10 @@
         <v>2.5</v>
       </c>
       <c r="C147" t="n">
-        <v>5</v>
+        <v>5.731037790654593</v>
       </c>
       <c r="D147" t="n">
-        <v>1.9</v>
+        <v>2.296073106391807</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3217,10 +3217,10 @@
         <v>3</v>
       </c>
       <c r="C148" t="n">
-        <v>5.2</v>
+        <v>5.73453898365369</v>
       </c>
       <c r="D148" t="n">
-        <v>2</v>
+        <v>2.289610904456333</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3236,10 +3236,10 @@
         <v>3.4</v>
       </c>
       <c r="C149" t="n">
-        <v>5.4</v>
+        <v>5.654270892304044</v>
       </c>
       <c r="D149" t="n">
-        <v>2.3</v>
+        <v>2.437762867347392</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>3</v>
       </c>
       <c r="C150" t="n">
-        <v>5.1</v>
+        <v>5.795615350415696</v>
       </c>
       <c r="D150" t="n">
-        <v>1.8</v>
+        <v>2.17688138180417</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(data): refaz iris_data_02 com escala+translacao (sem padrao diagonal)
Estrategia anterior (projecao ao longo do vetor normal) empurrava 72
amostras para o mesmo hiperplano, criando linha diagonal artificial.

Nova abordagem por classe:
  1. Escala em torno do centroide (fator 1.25) — aumenta dispersao interna
  2. Translacao rigida em sentidos opostos (1.10 cm em d_unit) — cria gap
  3. Clamping: petal_len [2.0, 7.5], petal_wid [0.4, 3.0]

Resultado: versicolor [2.00-4.34] x virginica [5.20-7.50] em petal_len
Gap de 0.86 cm em comprimento e 0.38 cm em largura de petala.
Clusters naturalmente dispersos, 0 erros pos-ajuste.
</commit_message>
<xml_diff>
--- a/data/iris_data_02.xlsx
+++ b/data/iris_data_02.xlsx
@@ -424,10 +424,10 @@
         <v>3.5</v>
       </c>
       <c r="C1" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D1" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E1" t="inlineStr">
         <is>
@@ -443,10 +443,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -462,10 +462,10 @@
         <v>3.2</v>
       </c>
       <c r="C3" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -481,10 +481,10 @@
         <v>3.1</v>
       </c>
       <c r="C4" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -500,10 +500,10 @@
         <v>3.6</v>
       </c>
       <c r="C5" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
         <v>3.9</v>
       </c>
       <c r="C6" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
         <v>0.4</v>
@@ -538,10 +538,10 @@
         <v>3.4</v>
       </c>
       <c r="C7" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -557,10 +557,10 @@
         <v>3.4</v>
       </c>
       <c r="C8" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -576,10 +576,10 @@
         <v>2.9</v>
       </c>
       <c r="C9" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -595,10 +595,10 @@
         <v>3.1</v>
       </c>
       <c r="C10" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -614,10 +614,10 @@
         <v>3.7</v>
       </c>
       <c r="C11" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -633,10 +633,10 @@
         <v>3.4</v>
       </c>
       <c r="C12" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -652,10 +652,10 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -671,10 +671,10 @@
         <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -690,10 +690,10 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         <v>4.4</v>
       </c>
       <c r="C16" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
         <v>0.4</v>
@@ -728,7 +728,7 @@
         <v>3.9</v>
       </c>
       <c r="C17" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
         <v>0.4</v>
@@ -747,10 +747,10 @@
         <v>3.5</v>
       </c>
       <c r="C18" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -766,10 +766,10 @@
         <v>3.8</v>
       </c>
       <c r="C19" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -785,10 +785,10 @@
         <v>3.8</v>
       </c>
       <c r="C20" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
         <v>3.4</v>
       </c>
       <c r="C21" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         <v>3.7</v>
       </c>
       <c r="C22" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D22" t="n">
         <v>0.4</v>
@@ -842,10 +842,10 @@
         <v>3.6</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -861,7 +861,7 @@
         <v>3.3</v>
       </c>
       <c r="C24" t="n">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
         <v>0.5</v>
@@ -880,10 +880,10 @@
         <v>3.4</v>
       </c>
       <c r="C25" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -899,10 +899,10 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         <v>3.4</v>
       </c>
       <c r="C27" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
         <v>0.4</v>
@@ -937,10 +937,10 @@
         <v>3.5</v>
       </c>
       <c r="C28" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -956,10 +956,10 @@
         <v>3.4</v>
       </c>
       <c r="C29" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -975,10 +975,10 @@
         <v>3.2</v>
       </c>
       <c r="C30" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -994,10 +994,10 @@
         <v>3.1</v>
       </c>
       <c r="C31" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>3.4</v>
       </c>
       <c r="C32" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
         <v>0.4</v>
@@ -1032,10 +1032,10 @@
         <v>4.1</v>
       </c>
       <c r="C33" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1051,10 +1051,10 @@
         <v>4.2</v>
       </c>
       <c r="C34" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1070,10 +1070,10 @@
         <v>3.1</v>
       </c>
       <c r="C35" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1089,10 +1089,10 @@
         <v>3.2</v>
       </c>
       <c r="C36" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1108,10 +1108,10 @@
         <v>3.5</v>
       </c>
       <c r="C37" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1127,10 +1127,10 @@
         <v>3.6</v>
       </c>
       <c r="C38" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1146,10 +1146,10 @@
         <v>3</v>
       </c>
       <c r="C39" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1165,10 +1165,10 @@
         <v>3.4</v>
       </c>
       <c r="C40" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1184,10 +1184,10 @@
         <v>3.5</v>
       </c>
       <c r="C41" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D41" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
         <v>2.3</v>
       </c>
       <c r="C42" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D42" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1222,10 +1222,10 @@
         <v>3.2</v>
       </c>
       <c r="C43" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         <v>3.5</v>
       </c>
       <c r="C44" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
         <v>0.6</v>
@@ -1260,7 +1260,7 @@
         <v>3.8</v>
       </c>
       <c r="C45" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="D45" t="n">
         <v>0.4</v>
@@ -1279,10 +1279,10 @@
         <v>3</v>
       </c>
       <c r="C46" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1298,10 +1298,10 @@
         <v>3.8</v>
       </c>
       <c r="C47" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1317,10 +1317,10 @@
         <v>3.2</v>
       </c>
       <c r="C48" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         <v>3.7</v>
       </c>
       <c r="C49" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>3.3</v>
       </c>
       <c r="C50" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="D50" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1374,10 +1374,10 @@
         <v>3.2</v>
       </c>
       <c r="C51" t="n">
-        <v>4.077326155578938</v>
+        <v>3.8428</v>
       </c>
       <c r="D51" t="n">
-        <v>1.062638009988589</v>
+        <v>0.8945</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>3.2</v>
       </c>
       <c r="C52" t="n">
-        <v>3.990055678231101</v>
+        <v>3.5928</v>
       </c>
       <c r="D52" t="n">
-        <v>1.223714376750597</v>
+        <v>1.0195</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1412,10 +1412,10 @@
         <v>3.1</v>
       </c>
       <c r="C53" t="n">
-        <v>4.080827348578034</v>
+        <v>4.0928</v>
       </c>
       <c r="D53" t="n">
-        <v>1.056175808053115</v>
+        <v>1.0195</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1431,10 +1431,10 @@
         <v>2.3</v>
       </c>
       <c r="C54" t="n">
-        <v>3.960360374646176</v>
+        <v>2.9678</v>
       </c>
       <c r="D54" t="n">
-        <v>1.278523422795916</v>
+        <v>0.7695</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1450,10 +1450,10 @@
         <v>2.8</v>
       </c>
       <c r="C55" t="n">
-        <v>4.012748595817834</v>
+        <v>3.7178</v>
       </c>
       <c r="D55" t="n">
-        <v>1.181829734576227</v>
+        <v>1.0195</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1469,10 +1469,10 @@
         <v>2.8</v>
       </c>
       <c r="C56" t="n">
-        <v>4.073824962579842</v>
+        <v>3.5928</v>
       </c>
       <c r="D56" t="n">
-        <v>1.069100211924063</v>
+        <v>0.7695</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1488,10 +1488,10 @@
         <v>3.3</v>
       </c>
       <c r="C57" t="n">
-        <v>3.993556871230197</v>
+        <v>3.8428</v>
       </c>
       <c r="D57" t="n">
-        <v>1.217252174815122</v>
+        <v>1.1445</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1507,10 +1507,10 @@
         <v>2.4</v>
       </c>
       <c r="C58" t="n">
-        <v>3.3</v>
+        <v>2.0928</v>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1526,10 +1526,10 @@
         <v>2.9</v>
       </c>
       <c r="C59" t="n">
-        <v>4.096517880166575</v>
+        <v>3.7178</v>
       </c>
       <c r="D59" t="n">
-        <v>1.027215569749693</v>
+        <v>0.7695</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1545,10 +1545,10 @@
         <v>2.7</v>
       </c>
       <c r="C60" t="n">
-        <v>3.895782814885072</v>
+        <v>2.8428</v>
       </c>
       <c r="D60" t="n">
-        <v>1.397715147383553</v>
+        <v>0.8945</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1564,10 +1564,10 @@
         <v>2</v>
       </c>
       <c r="C61" t="n">
-        <v>3.5</v>
+        <v>2.3428</v>
       </c>
       <c r="D61" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1583,10 +1583,10 @@
         <v>3</v>
       </c>
       <c r="C62" t="n">
-        <v>3.921976925470902</v>
+        <v>3.2178</v>
       </c>
       <c r="D62" t="n">
-        <v>1.349368303273708</v>
+        <v>1.0195</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1602,10 +1602,10 @@
         <v>2.2</v>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>2.9678</v>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         <v>2.9</v>
       </c>
       <c r="C64" t="n">
-        <v>4.077326155578938</v>
+        <v>3.8428</v>
       </c>
       <c r="D64" t="n">
-        <v>1.062638009988589</v>
+        <v>0.8945</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1640,10 +1640,10 @@
         <v>2.9</v>
       </c>
       <c r="C65" t="n">
-        <v>3.6</v>
+        <v>2.4678</v>
       </c>
       <c r="D65" t="n">
-        <v>1.3</v>
+        <v>0.7695</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1659,10 +1659,10 @@
         <v>3.1</v>
       </c>
       <c r="C66" t="n">
-        <v>4.009247402818739</v>
+        <v>3.4678</v>
       </c>
       <c r="D66" t="n">
-        <v>1.1882919365117</v>
+        <v>0.8945</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1678,10 +1678,10 @@
         <v>3</v>
       </c>
       <c r="C67" t="n">
-        <v>3.990055678231101</v>
+        <v>3.5928</v>
       </c>
       <c r="D67" t="n">
-        <v>1.223714376750597</v>
+        <v>1.0195</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1697,10 +1697,10 @@
         <v>2.7</v>
       </c>
       <c r="C68" t="n">
-        <v>4.1</v>
+        <v>3.0928</v>
       </c>
       <c r="D68" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1716,10 +1716,10 @@
         <v>2.2</v>
       </c>
       <c r="C69" t="n">
-        <v>3.990055678231101</v>
+        <v>3.5928</v>
       </c>
       <c r="D69" t="n">
-        <v>1.223714376750597</v>
+        <v>1.0195</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1735,10 +1735,10 @@
         <v>2.5</v>
       </c>
       <c r="C70" t="n">
-        <v>3.9</v>
+        <v>2.8428</v>
       </c>
       <c r="D70" t="n">
-        <v>1.1</v>
+        <v>0.5195</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -1754,10 +1754,10 @@
         <v>3.2</v>
       </c>
       <c r="C71" t="n">
-        <v>3.932480504468189</v>
+        <v>3.9678</v>
       </c>
       <c r="D71" t="n">
-        <v>1.329981697467285</v>
+        <v>1.3945</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -1773,10 +1773,10 @@
         <v>2.8</v>
       </c>
       <c r="C72" t="n">
-        <v>3.960360374646176</v>
+        <v>2.9678</v>
       </c>
       <c r="D72" t="n">
-        <v>1.278523422795916</v>
+        <v>0.7695</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -1792,10 +1792,10 @@
         <v>2.5</v>
       </c>
       <c r="C73" t="n">
-        <v>4.080827348578034</v>
+        <v>4.0928</v>
       </c>
       <c r="D73" t="n">
-        <v>1.056175808053115</v>
+        <v>1.0195</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -1811,10 +1811,10 @@
         <v>2.8</v>
       </c>
       <c r="C74" t="n">
-        <v>4.16109543992768</v>
+        <v>3.8428</v>
       </c>
       <c r="D74" t="n">
-        <v>0.9080238451620553</v>
+        <v>0.6445</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -1830,10 +1830,10 @@
         <v>2.9</v>
       </c>
       <c r="C75" t="n">
-        <v>4.028439127406376</v>
+        <v>3.3428</v>
       </c>
       <c r="D75" t="n">
-        <v>1.152869496272804</v>
+        <v>0.7695</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -1849,10 +1849,10 @@
         <v>3</v>
       </c>
       <c r="C76" t="n">
-        <v>4.009247402818739</v>
+        <v>3.4678</v>
       </c>
       <c r="D76" t="n">
-        <v>1.1882919365117</v>
+        <v>0.8945</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1868,10 +1868,10 @@
         <v>2.8</v>
       </c>
       <c r="C77" t="n">
-        <v>4.100019073165671</v>
+        <v>3.9678</v>
       </c>
       <c r="D77" t="n">
-        <v>1.020753367814218</v>
+        <v>0.8945</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -1887,10 +1887,10 @@
         <v>3</v>
       </c>
       <c r="C78" t="n">
-        <v>4.019750981816026</v>
+        <v>4.2178</v>
       </c>
       <c r="D78" t="n">
-        <v>1.168905330705277</v>
+        <v>1.2695</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1906,10 +1906,10 @@
         <v>2.9</v>
       </c>
       <c r="C79" t="n">
-        <v>3.990055678231101</v>
+        <v>3.5928</v>
       </c>
       <c r="D79" t="n">
-        <v>1.223714376750597</v>
+        <v>1.0195</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1925,10 +1925,10 @@
         <v>2.6</v>
       </c>
       <c r="C80" t="n">
-        <v>3.5</v>
+        <v>2.3428</v>
       </c>
       <c r="D80" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1944,10 +1944,10 @@
         <v>2.4</v>
       </c>
       <c r="C81" t="n">
-        <v>3.8</v>
+        <v>2.7178</v>
       </c>
       <c r="D81" t="n">
-        <v>1.1</v>
+        <v>0.5195</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1963,10 +1963,10 @@
         <v>2.4</v>
       </c>
       <c r="C82" t="n">
-        <v>3.7</v>
+        <v>2.5928</v>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -1982,10 +1982,10 @@
         <v>2.7</v>
       </c>
       <c r="C83" t="n">
-        <v>3.9</v>
+        <v>2.8428</v>
       </c>
       <c r="D83" t="n">
-        <v>1.2</v>
+        <v>0.6445</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2001,10 +2001,10 @@
         <v>2.7</v>
       </c>
       <c r="C84" t="n">
-        <v>4.084328541577129</v>
+        <v>4.3428</v>
       </c>
       <c r="D84" t="n">
-        <v>1.049713606117641</v>
+        <v>1.1445</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2020,10 +2020,10 @@
         <v>3</v>
       </c>
       <c r="C85" t="n">
-        <v>3.990055678231101</v>
+        <v>3.5928</v>
       </c>
       <c r="D85" t="n">
-        <v>1.223714376750597</v>
+        <v>1.0195</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2039,10 +2039,10 @@
         <v>3.4</v>
       </c>
       <c r="C86" t="n">
-        <v>3.94817103605673</v>
+        <v>3.5928</v>
       </c>
       <c r="D86" t="n">
-        <v>1.301021459163863</v>
+        <v>1.1445</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2058,10 +2058,10 @@
         <v>3.1</v>
       </c>
       <c r="C87" t="n">
-        <v>4.035441513404567</v>
+        <v>3.8428</v>
       </c>
       <c r="D87" t="n">
-        <v>1.139945092401856</v>
+        <v>1.0195</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2077,10 +2077,10 @@
         <v>2.3</v>
       </c>
       <c r="C88" t="n">
-        <v>4.051132044993109</v>
+        <v>3.4678</v>
       </c>
       <c r="D88" t="n">
-        <v>1.110984854098434</v>
+        <v>0.7695</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2096,10 +2096,10 @@
         <v>3</v>
       </c>
       <c r="C89" t="n">
-        <v>3.983053292232909</v>
+        <v>3.0928</v>
       </c>
       <c r="D89" t="n">
-        <v>1.236638780621545</v>
+        <v>0.7695</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2115,10 +2115,10 @@
         <v>2.5</v>
       </c>
       <c r="C90" t="n">
-        <v>3.960360374646176</v>
+        <v>2.9678</v>
       </c>
       <c r="D90" t="n">
-        <v>1.278523422795916</v>
+        <v>0.7695</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2134,10 +2134,10 @@
         <v>2.6</v>
       </c>
       <c r="C91" t="n">
-        <v>4.09301668716748</v>
+        <v>3.4678</v>
       </c>
       <c r="D91" t="n">
-        <v>1.033677771685167</v>
+        <v>0.6445</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2153,10 +2153,10 @@
         <v>3</v>
       </c>
       <c r="C92" t="n">
-        <v>4.054633237992205</v>
+        <v>3.7178</v>
       </c>
       <c r="D92" t="n">
-        <v>1.10452265216296</v>
+        <v>0.8945</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2172,10 +2172,10 @@
         <v>2.6</v>
       </c>
       <c r="C93" t="n">
-        <v>4</v>
+        <v>2.9678</v>
       </c>
       <c r="D93" t="n">
-        <v>1.2</v>
+        <v>0.6445</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2191,10 +2191,10 @@
         <v>2.3</v>
       </c>
       <c r="C94" t="n">
-        <v>3.3</v>
+        <v>2.0928</v>
       </c>
       <c r="D94" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2210,10 +2210,10 @@
         <v>2.7</v>
       </c>
       <c r="C95" t="n">
-        <v>4.005746209819643</v>
+        <v>3.2178</v>
       </c>
       <c r="D95" t="n">
-        <v>1.194754138447175</v>
+        <v>0.7695</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2229,10 +2229,10 @@
         <v>3</v>
       </c>
       <c r="C96" t="n">
-        <v>4.047630851994013</v>
+        <v>3.2178</v>
       </c>
       <c r="D96" t="n">
-        <v>1.117447056033908</v>
+        <v>0.6445</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>2.9</v>
       </c>
       <c r="C97" t="n">
-        <v>4.005746209819643</v>
+        <v>3.2178</v>
       </c>
       <c r="D97" t="n">
-        <v>1.194754138447175</v>
+        <v>0.7695</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2267,10 +2267,10 @@
         <v>2.9</v>
       </c>
       <c r="C98" t="n">
-        <v>4.028439127406376</v>
+        <v>3.3428</v>
       </c>
       <c r="D98" t="n">
-        <v>1.152869496272804</v>
+        <v>0.7695</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2286,10 +2286,10 @@
         <v>2.5</v>
       </c>
       <c r="C99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D99" t="n">
-        <v>1.1</v>
+        <v>0.5195</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2305,10 +2305,10 @@
         <v>2.8</v>
       </c>
       <c r="C100" t="n">
-        <v>3.983053292232909</v>
+        <v>3.0928</v>
       </c>
       <c r="D100" t="n">
-        <v>1.236638780621545</v>
+        <v>0.7695</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2324,10 +2324,10 @@
         <v>3.3</v>
       </c>
       <c r="C101" t="n">
-        <v>6</v>
+        <v>7.0792</v>
       </c>
       <c r="D101" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2343,10 +2343,10 @@
         <v>2.7</v>
       </c>
       <c r="C102" t="n">
-        <v>5.753730708241326</v>
+        <v>5.9542</v>
       </c>
       <c r="D102" t="n">
-        <v>2.254188464217437</v>
+        <v>2.3925</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2362,10 +2362,10 @@
         <v>3</v>
       </c>
       <c r="C103" t="n">
-        <v>5.9</v>
+        <v>6.9542</v>
       </c>
       <c r="D103" t="n">
-        <v>2.1</v>
+        <v>2.6425</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2381,10 +2381,10 @@
         <v>2.9</v>
       </c>
       <c r="C104" t="n">
-        <v>5.909079938349363</v>
+        <v>6.5792</v>
       </c>
       <c r="D104" t="n">
-        <v>1.967458170932317</v>
+        <v>2.2675</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2400,10 +2400,10 @@
         <v>3</v>
       </c>
       <c r="C105" t="n">
-        <v>5.8</v>
+        <v>6.8292</v>
       </c>
       <c r="D105" t="n">
-        <v>2.2</v>
+        <v>2.7675</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2419,10 +2419,10 @@
         <v>3</v>
       </c>
       <c r="C106" t="n">
-        <v>6.6</v>
+        <v>7.5</v>
       </c>
       <c r="D106" t="n">
-        <v>2.1</v>
+        <v>2.6425</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2438,10 +2438,10 @@
         <v>2.5</v>
       </c>
       <c r="C107" t="n">
-        <v>5.701342487069668</v>
+        <v>5.2042</v>
       </c>
       <c r="D107" t="n">
-        <v>2.350882152437126</v>
+        <v>2.1425</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2457,10 +2457,10 @@
         <v>2.9</v>
       </c>
       <c r="C108" t="n">
-        <v>6.3</v>
+        <v>7.4542</v>
       </c>
       <c r="D108" t="n">
-        <v>1.8</v>
+        <v>2.2675</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2476,10 +2476,10 @@
         <v>2.5</v>
       </c>
       <c r="C109" t="n">
-        <v>5.954465773522829</v>
+        <v>6.8292</v>
       </c>
       <c r="D109" t="n">
-        <v>1.883688886583576</v>
+        <v>2.2675</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2495,10 +2495,10 @@
         <v>3.6</v>
       </c>
       <c r="C110" t="n">
-        <v>6.1</v>
+        <v>7.2042</v>
       </c>
       <c r="D110" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2514,10 +2514,10 @@
         <v>3.2</v>
       </c>
       <c r="C111" t="n">
-        <v>5.711846066066955</v>
+        <v>5.9542</v>
       </c>
       <c r="D111" t="n">
-        <v>2.331495546630703</v>
+        <v>2.5175</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2533,10 +2533,10 @@
         <v>2.7</v>
       </c>
       <c r="C112" t="n">
-        <v>5.799116543414793</v>
+        <v>6.2042</v>
       </c>
       <c r="D112" t="n">
-        <v>2.170419179868695</v>
+        <v>2.3925</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2552,10 +2552,10 @@
         <v>3</v>
       </c>
       <c r="C113" t="n">
-        <v>5.760733094239518</v>
+        <v>6.4542</v>
       </c>
       <c r="D113" t="n">
-        <v>2.241264060346488</v>
+        <v>2.6425</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2571,10 +2571,10 @@
         <v>2.5</v>
       </c>
       <c r="C114" t="n">
-        <v>5.689153148480223</v>
+        <v>5.8292</v>
       </c>
       <c r="D114" t="n">
-        <v>2.373380188805074</v>
+        <v>2.5175</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2590,10 +2590,10 @@
         <v>2.8</v>
       </c>
       <c r="C115" t="n">
-        <v>5.544307497369473</v>
+        <v>5.9542</v>
       </c>
       <c r="D115" t="n">
-        <v>2.64072387628377</v>
+        <v>3</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2609,10 +2609,10 @@
         <v>3.2</v>
       </c>
       <c r="C116" t="n">
-        <v>5.631577974717311</v>
+        <v>6.2042</v>
       </c>
       <c r="D116" t="n">
-        <v>2.479647509521762</v>
+        <v>2.8925</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -2628,10 +2628,10 @@
         <v>3</v>
       </c>
       <c r="C117" t="n">
-        <v>5.88638702076263</v>
+        <v>6.4542</v>
       </c>
       <c r="D117" t="n">
-        <v>2.009342813106688</v>
+        <v>2.2675</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -2647,10 +2647,10 @@
         <v>3.8</v>
       </c>
       <c r="C118" t="n">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="D118" t="n">
-        <v>2.2</v>
+        <v>2.7675</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -2666,10 +2666,10 @@
         <v>2.6</v>
       </c>
       <c r="C119" t="n">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="D119" t="n">
-        <v>2.3</v>
+        <v>2.8925</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -2685,10 +2685,10 @@
         <v>2.2</v>
       </c>
       <c r="C120" t="n">
-        <v>5.898576359352075</v>
+        <v>5.8292</v>
       </c>
       <c r="D120" t="n">
-        <v>1.98684477673874</v>
+        <v>1.8925</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -2704,10 +2704,10 @@
         <v>3.2</v>
       </c>
       <c r="C121" t="n">
-        <v>5.722349645064243</v>
+        <v>6.7042</v>
       </c>
       <c r="D121" t="n">
-        <v>2.31210894082428</v>
+        <v>2.8925</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -2723,10 +2723,10 @@
         <v>2.8</v>
       </c>
       <c r="C122" t="n">
-        <v>5.666460230893489</v>
+        <v>5.7042</v>
       </c>
       <c r="D122" t="n">
-        <v>2.415264830979444</v>
+        <v>2.5175</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -2742,10 +2742,10 @@
         <v>2.8</v>
       </c>
       <c r="C123" t="n">
-        <v>6.7</v>
+        <v>7.5</v>
       </c>
       <c r="D123" t="n">
-        <v>2</v>
+        <v>2.5175</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2761,10 +2761,10 @@
         <v>2.7</v>
       </c>
       <c r="C124" t="n">
-        <v>5.75022951524223</v>
+        <v>5.7042</v>
       </c>
       <c r="D124" t="n">
-        <v>2.260650666152911</v>
+        <v>2.2675</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2780,10 +2780,10 @@
         <v>3.3</v>
       </c>
       <c r="C125" t="n">
-        <v>5.806118929412984</v>
+        <v>6.7042</v>
       </c>
       <c r="D125" t="n">
-        <v>2.157494775997747</v>
+        <v>2.6425</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2799,10 +2799,10 @@
         <v>3.2</v>
       </c>
       <c r="C126" t="n">
-        <v>6</v>
+        <v>7.0792</v>
       </c>
       <c r="D126" t="n">
-        <v>1.8</v>
+        <v>2.2675</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -2818,10 +2818,10 @@
         <v>2.8</v>
       </c>
       <c r="C127" t="n">
-        <v>5.727536597655497</v>
+        <v>5.5792</v>
       </c>
       <c r="D127" t="n">
-        <v>2.302535308327282</v>
+        <v>2.2675</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -2837,10 +2837,10 @@
         <v>3</v>
       </c>
       <c r="C128" t="n">
-        <v>5.75022951524223</v>
+        <v>5.7042</v>
       </c>
       <c r="D128" t="n">
-        <v>2.260650666152911</v>
+        <v>2.2675</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2856,10 +2856,10 @@
         <v>2.8</v>
       </c>
       <c r="C129" t="n">
-        <v>5.783426011826251</v>
+        <v>6.5792</v>
       </c>
       <c r="D129" t="n">
-        <v>2.199379418172118</v>
+        <v>2.6425</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -2875,10 +2875,10 @@
         <v>3</v>
       </c>
       <c r="C130" t="n">
-        <v>6.038235057871571</v>
+        <v>6.8292</v>
       </c>
       <c r="D130" t="n">
-        <v>1.729074721757043</v>
+        <v>2.0175</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -2894,10 +2894,10 @@
         <v>2.8</v>
       </c>
       <c r="C131" t="n">
-        <v>6.1</v>
+        <v>7.2042</v>
       </c>
       <c r="D131" t="n">
-        <v>1.9</v>
+        <v>2.3925</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -2913,10 +2913,10 @@
         <v>3.8</v>
       </c>
       <c r="C132" t="n">
-        <v>6.4</v>
+        <v>7.5</v>
       </c>
       <c r="D132" t="n">
-        <v>2</v>
+        <v>2.5175</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -2932,10 +2932,10 @@
         <v>2.8</v>
       </c>
       <c r="C133" t="n">
-        <v>5.74154136965188</v>
+        <v>6.5792</v>
       </c>
       <c r="D133" t="n">
-        <v>2.276686500585384</v>
+        <v>2.7675</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -2951,10 +2951,10 @@
         <v>2.8</v>
       </c>
       <c r="C134" t="n">
-        <v>5.921269276938808</v>
+        <v>5.9542</v>
       </c>
       <c r="D134" t="n">
-        <v>1.94496013456437</v>
+        <v>1.8925</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2970,10 +2970,10 @@
         <v>2.6</v>
       </c>
       <c r="C135" t="n">
-        <v>6.076618507046845</v>
+        <v>6.5792</v>
       </c>
       <c r="D135" t="n">
-        <v>1.65822984127925</v>
+        <v>1.7675</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -2989,10 +2989,10 @@
         <v>3</v>
       </c>
       <c r="C136" t="n">
-        <v>6.1</v>
+        <v>7.2042</v>
       </c>
       <c r="D136" t="n">
-        <v>2.3</v>
+        <v>2.8925</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3008,10 +3008,10 @@
         <v>3.4</v>
       </c>
       <c r="C137" t="n">
-        <v>5.657772085303139</v>
+        <v>6.5792</v>
       </c>
       <c r="D137" t="n">
-        <v>2.431300665411918</v>
+        <v>3</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3027,10 +3027,10 @@
         <v>3.1</v>
       </c>
       <c r="C138" t="n">
-        <v>5.88638702076263</v>
+        <v>6.4542</v>
       </c>
       <c r="D138" t="n">
-        <v>2.009342813106688</v>
+        <v>2.2675</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3046,10 +3046,10 @@
         <v>3</v>
       </c>
       <c r="C139" t="n">
-        <v>5.727536597655497</v>
+        <v>5.5792</v>
       </c>
       <c r="D139" t="n">
-        <v>2.302535308327282</v>
+        <v>2.2675</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3065,10 +3065,10 @@
         <v>3.1</v>
       </c>
       <c r="C140" t="n">
-        <v>5.738040176652785</v>
+        <v>6.3292</v>
       </c>
       <c r="D140" t="n">
-        <v>2.283148702520858</v>
+        <v>2.6425</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3084,10 +3084,10 @@
         <v>3.1</v>
       </c>
       <c r="C141" t="n">
-        <v>5.657772085303139</v>
+        <v>6.5792</v>
       </c>
       <c r="D141" t="n">
-        <v>2.431300665411918</v>
+        <v>3</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3103,10 +3103,10 @@
         <v>3.1</v>
       </c>
       <c r="C142" t="n">
-        <v>5.586192139543845</v>
+        <v>5.9542</v>
       </c>
       <c r="D142" t="n">
-        <v>2.563416793870504</v>
+        <v>2.8925</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3122,10 +3122,10 @@
         <v>2.7</v>
       </c>
       <c r="C143" t="n">
-        <v>5.753730708241326</v>
+        <v>5.9542</v>
       </c>
       <c r="D143" t="n">
-        <v>2.254188464217437</v>
+        <v>2.3925</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3141,10 +3141,10 @@
         <v>3.2</v>
       </c>
       <c r="C144" t="n">
-        <v>5.9</v>
+        <v>6.9542</v>
       </c>
       <c r="D144" t="n">
-        <v>2.3</v>
+        <v>2.8925</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3160,10 +3160,10 @@
         <v>3.3</v>
       </c>
       <c r="C145" t="n">
-        <v>5.7</v>
+        <v>6.7042</v>
       </c>
       <c r="D145" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3179,10 +3179,10 @@
         <v>3</v>
       </c>
       <c r="C146" t="n">
-        <v>5.608885057130578</v>
+        <v>6.0792</v>
       </c>
       <c r="D146" t="n">
-        <v>2.521532151696133</v>
+        <v>2.8925</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3198,10 +3198,10 @@
         <v>2.5</v>
       </c>
       <c r="C147" t="n">
-        <v>5.731037790654593</v>
+        <v>5.8292</v>
       </c>
       <c r="D147" t="n">
-        <v>2.296073106391807</v>
+        <v>2.3925</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3217,10 +3217,10 @@
         <v>3</v>
       </c>
       <c r="C148" t="n">
-        <v>5.73453898365369</v>
+        <v>6.0792</v>
       </c>
       <c r="D148" t="n">
-        <v>2.289610904456333</v>
+        <v>2.5175</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3236,10 +3236,10 @@
         <v>3.4</v>
       </c>
       <c r="C149" t="n">
-        <v>5.654270892304044</v>
+        <v>6.3292</v>
       </c>
       <c r="D149" t="n">
-        <v>2.437762867347392</v>
+        <v>2.8925</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>3</v>
       </c>
       <c r="C150" t="n">
-        <v>5.795615350415696</v>
+        <v>5.9542</v>
       </c>
       <c r="D150" t="n">
-        <v>2.17688138180417</v>
+        <v>2.2675</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(data): iris_data_02 com ajuste minimo (9 amostras, ~0.08 cm)
Volta para abordagem minimalista: apenas as 9 amostras que cruzam
a fronteira ver x vir sao deslocadas pelo minimo necessario (margem
0.12 no espaco discriminante ~= 0.08 cm fisico). Os 141 demais pontos
sao identicos ao dataset original. Gap visual sutil, sem distancia
exagerada entre os clusters.
</commit_message>
<xml_diff>
--- a/data/iris_data_02.xlsx
+++ b/data/iris_data_02.xlsx
@@ -424,10 +424,10 @@
         <v>3.5</v>
       </c>
       <c r="C1" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D1" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E1" t="inlineStr">
         <is>
@@ -443,10 +443,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -462,10 +462,10 @@
         <v>3.2</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -481,10 +481,10 @@
         <v>3.1</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -500,10 +500,10 @@
         <v>3.6</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
         <v>3.9</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="D6" t="n">
         <v>0.4</v>
@@ -538,10 +538,10 @@
         <v>3.4</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -557,10 +557,10 @@
         <v>3.4</v>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -576,10 +576,10 @@
         <v>2.9</v>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D9" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -595,10 +595,10 @@
         <v>3.1</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D10" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -614,10 +614,10 @@
         <v>3.7</v>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D11" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -633,10 +633,10 @@
         <v>3.4</v>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="D12" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -652,10 +652,10 @@
         <v>3</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D13" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -671,10 +671,10 @@
         <v>3</v>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>1.1</v>
       </c>
       <c r="D14" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -690,10 +690,10 @@
         <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         <v>4.4</v>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D16" t="n">
         <v>0.4</v>
@@ -728,7 +728,7 @@
         <v>3.9</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D17" t="n">
         <v>0.4</v>
@@ -747,10 +747,10 @@
         <v>3.5</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D18" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -766,10 +766,10 @@
         <v>3.8</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -785,10 +785,10 @@
         <v>3.8</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D20" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
         <v>3.4</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="D21" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         <v>3.7</v>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D22" t="n">
         <v>0.4</v>
@@ -842,10 +842,10 @@
         <v>3.6</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -861,7 +861,7 @@
         <v>3.3</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="D24" t="n">
         <v>0.5</v>
@@ -880,10 +880,10 @@
         <v>3.4</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="D25" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -899,10 +899,10 @@
         <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="D26" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -918,7 +918,7 @@
         <v>3.4</v>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="D27" t="n">
         <v>0.4</v>
@@ -937,10 +937,10 @@
         <v>3.5</v>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D28" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -956,10 +956,10 @@
         <v>3.4</v>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D29" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -975,10 +975,10 @@
         <v>3.2</v>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="D30" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -994,10 +994,10 @@
         <v>3.1</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="D31" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>3.4</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D32" t="n">
         <v>0.4</v>
@@ -1032,10 +1032,10 @@
         <v>4.1</v>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D33" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1051,10 +1051,10 @@
         <v>4.2</v>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D34" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1070,10 +1070,10 @@
         <v>3.1</v>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D35" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1089,10 +1089,10 @@
         <v>3.2</v>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="D36" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1108,10 +1108,10 @@
         <v>3.5</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D37" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1127,10 +1127,10 @@
         <v>3.6</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D38" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1146,10 +1146,10 @@
         <v>3</v>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D39" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1165,10 +1165,10 @@
         <v>3.4</v>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D40" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1184,10 +1184,10 @@
         <v>3.5</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D41" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
         <v>2.3</v>
       </c>
       <c r="C42" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D42" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1222,10 +1222,10 @@
         <v>3.2</v>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="D43" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         <v>3.5</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="D44" t="n">
         <v>0.6</v>
@@ -1260,7 +1260,7 @@
         <v>3.8</v>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="D45" t="n">
         <v>0.4</v>
@@ -1279,10 +1279,10 @@
         <v>3</v>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D46" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1298,10 +1298,10 @@
         <v>3.8</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="D47" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1317,10 +1317,10 @@
         <v>3.2</v>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D48" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         <v>3.7</v>
       </c>
       <c r="C49" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D49" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>3.3</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="D50" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1374,10 +1374,10 @@
         <v>3.2</v>
       </c>
       <c r="C51" t="n">
-        <v>3.8428</v>
+        <v>4.7</v>
       </c>
       <c r="D51" t="n">
-        <v>0.8945</v>
+        <v>1.4</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>3.2</v>
       </c>
       <c r="C52" t="n">
-        <v>3.5928</v>
+        <v>4.5</v>
       </c>
       <c r="D52" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1412,10 +1412,10 @@
         <v>3.1</v>
       </c>
       <c r="C53" t="n">
-        <v>4.0928</v>
+        <v>4.9</v>
       </c>
       <c r="D53" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1431,10 +1431,10 @@
         <v>2.3</v>
       </c>
       <c r="C54" t="n">
-        <v>2.9678</v>
+        <v>4</v>
       </c>
       <c r="D54" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1450,10 +1450,10 @@
         <v>2.8</v>
       </c>
       <c r="C55" t="n">
-        <v>3.7178</v>
+        <v>4.6</v>
       </c>
       <c r="D55" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1469,10 +1469,10 @@
         <v>2.8</v>
       </c>
       <c r="C56" t="n">
-        <v>3.5928</v>
+        <v>4.5</v>
       </c>
       <c r="D56" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1488,10 +1488,10 @@
         <v>3.3</v>
       </c>
       <c r="C57" t="n">
-        <v>3.8428</v>
+        <v>4.7</v>
       </c>
       <c r="D57" t="n">
-        <v>1.1445</v>
+        <v>1.6</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1507,10 +1507,10 @@
         <v>2.4</v>
       </c>
       <c r="C58" t="n">
-        <v>2.0928</v>
+        <v>3.3</v>
       </c>
       <c r="D58" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1526,10 +1526,10 @@
         <v>2.9</v>
       </c>
       <c r="C59" t="n">
-        <v>3.7178</v>
+        <v>4.6</v>
       </c>
       <c r="D59" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1545,10 +1545,10 @@
         <v>2.7</v>
       </c>
       <c r="C60" t="n">
-        <v>2.8428</v>
+        <v>3.9</v>
       </c>
       <c r="D60" t="n">
-        <v>0.8945</v>
+        <v>1.4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1564,10 +1564,10 @@
         <v>2</v>
       </c>
       <c r="C61" t="n">
-        <v>2.3428</v>
+        <v>3.5</v>
       </c>
       <c r="D61" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1583,10 +1583,10 @@
         <v>3</v>
       </c>
       <c r="C62" t="n">
-        <v>3.2178</v>
+        <v>4.2</v>
       </c>
       <c r="D62" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1602,10 +1602,10 @@
         <v>2.2</v>
       </c>
       <c r="C63" t="n">
-        <v>2.9678</v>
+        <v>4</v>
       </c>
       <c r="D63" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         <v>2.9</v>
       </c>
       <c r="C64" t="n">
-        <v>3.8428</v>
+        <v>4.7</v>
       </c>
       <c r="D64" t="n">
-        <v>0.8945</v>
+        <v>1.4</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1640,10 +1640,10 @@
         <v>2.9</v>
       </c>
       <c r="C65" t="n">
-        <v>2.4678</v>
+        <v>3.6</v>
       </c>
       <c r="D65" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1659,10 +1659,10 @@
         <v>3.1</v>
       </c>
       <c r="C66" t="n">
-        <v>3.4678</v>
+        <v>4.4</v>
       </c>
       <c r="D66" t="n">
-        <v>0.8945</v>
+        <v>1.4</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1678,10 +1678,10 @@
         <v>3</v>
       </c>
       <c r="C67" t="n">
-        <v>3.5928</v>
+        <v>4.5</v>
       </c>
       <c r="D67" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1697,10 +1697,10 @@
         <v>2.7</v>
       </c>
       <c r="C68" t="n">
-        <v>3.0928</v>
+        <v>4.1</v>
       </c>
       <c r="D68" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1716,10 +1716,10 @@
         <v>2.2</v>
       </c>
       <c r="C69" t="n">
-        <v>3.5928</v>
+        <v>4.5</v>
       </c>
       <c r="D69" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1735,10 +1735,10 @@
         <v>2.5</v>
       </c>
       <c r="C70" t="n">
-        <v>2.8428</v>
+        <v>3.9</v>
       </c>
       <c r="D70" t="n">
-        <v>0.5195</v>
+        <v>1.1</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -1754,10 +1754,10 @@
         <v>3.2</v>
       </c>
       <c r="C71" t="n">
-        <v>3.9678</v>
+        <v>4.7582</v>
       </c>
       <c r="D71" t="n">
-        <v>1.3945</v>
+        <v>1.7774</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -1773,10 +1773,10 @@
         <v>2.8</v>
       </c>
       <c r="C72" t="n">
-        <v>2.9678</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -1792,10 +1792,10 @@
         <v>2.5</v>
       </c>
       <c r="C73" t="n">
-        <v>4.0928</v>
+        <v>4.9</v>
       </c>
       <c r="D73" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -1811,10 +1811,10 @@
         <v>2.8</v>
       </c>
       <c r="C74" t="n">
-        <v>3.8428</v>
+        <v>4.7</v>
       </c>
       <c r="D74" t="n">
-        <v>0.6445</v>
+        <v>1.2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -1830,10 +1830,10 @@
         <v>2.9</v>
       </c>
       <c r="C75" t="n">
-        <v>3.3428</v>
+        <v>4.3</v>
       </c>
       <c r="D75" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -1849,10 +1849,10 @@
         <v>3</v>
       </c>
       <c r="C76" t="n">
-        <v>3.4678</v>
+        <v>4.4</v>
       </c>
       <c r="D76" t="n">
-        <v>0.8945</v>
+        <v>1.4</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -1868,10 +1868,10 @@
         <v>2.8</v>
       </c>
       <c r="C77" t="n">
-        <v>3.9678</v>
+        <v>4.8</v>
       </c>
       <c r="D77" t="n">
-        <v>0.8945</v>
+        <v>1.4</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -1887,10 +1887,10 @@
         <v>3</v>
       </c>
       <c r="C78" t="n">
-        <v>4.2178</v>
+        <v>4.8455</v>
       </c>
       <c r="D78" t="n">
-        <v>1.2695</v>
+        <v>1.6163</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -1906,10 +1906,10 @@
         <v>2.9</v>
       </c>
       <c r="C79" t="n">
-        <v>3.5928</v>
+        <v>4.5</v>
       </c>
       <c r="D79" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -1925,10 +1925,10 @@
         <v>2.6</v>
       </c>
       <c r="C80" t="n">
-        <v>2.3428</v>
+        <v>3.5</v>
       </c>
       <c r="D80" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -1944,10 +1944,10 @@
         <v>2.4</v>
       </c>
       <c r="C81" t="n">
-        <v>2.7178</v>
+        <v>3.8</v>
       </c>
       <c r="D81" t="n">
-        <v>0.5195</v>
+        <v>1.1</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -1963,10 +1963,10 @@
         <v>2.4</v>
       </c>
       <c r="C82" t="n">
-        <v>2.5928</v>
+        <v>3.7</v>
       </c>
       <c r="D82" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -1982,10 +1982,10 @@
         <v>2.7</v>
       </c>
       <c r="C83" t="n">
-        <v>2.8428</v>
+        <v>3.9</v>
       </c>
       <c r="D83" t="n">
-        <v>0.6445</v>
+        <v>1.2</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2001,10 +2001,10 @@
         <v>2.7</v>
       </c>
       <c r="C84" t="n">
-        <v>4.3428</v>
+        <v>4.9101</v>
       </c>
       <c r="D84" t="n">
-        <v>1.1445</v>
+        <v>1.4971</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2020,10 +2020,10 @@
         <v>3</v>
       </c>
       <c r="C85" t="n">
-        <v>3.5928</v>
+        <v>4.5</v>
       </c>
       <c r="D85" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2039,10 +2039,10 @@
         <v>3.4</v>
       </c>
       <c r="C86" t="n">
-        <v>3.5928</v>
+        <v>4.5</v>
       </c>
       <c r="D86" t="n">
-        <v>1.1445</v>
+        <v>1.6</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2058,10 +2058,10 @@
         <v>3.1</v>
       </c>
       <c r="C87" t="n">
-        <v>3.8428</v>
+        <v>4.7</v>
       </c>
       <c r="D87" t="n">
-        <v>1.0195</v>
+        <v>1.5</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2077,10 +2077,10 @@
         <v>2.3</v>
       </c>
       <c r="C88" t="n">
-        <v>3.4678</v>
+        <v>4.4</v>
       </c>
       <c r="D88" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2096,10 +2096,10 @@
         <v>3</v>
       </c>
       <c r="C89" t="n">
-        <v>3.0928</v>
+        <v>4.1</v>
       </c>
       <c r="D89" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2115,10 +2115,10 @@
         <v>2.5</v>
       </c>
       <c r="C90" t="n">
-        <v>2.9678</v>
+        <v>4</v>
       </c>
       <c r="D90" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2134,10 +2134,10 @@
         <v>2.6</v>
       </c>
       <c r="C91" t="n">
-        <v>3.4678</v>
+        <v>4.4</v>
       </c>
       <c r="D91" t="n">
-        <v>0.6445</v>
+        <v>1.2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2153,10 +2153,10 @@
         <v>3</v>
       </c>
       <c r="C92" t="n">
-        <v>3.7178</v>
+        <v>4.6</v>
       </c>
       <c r="D92" t="n">
-        <v>0.8945</v>
+        <v>1.4</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2172,10 +2172,10 @@
         <v>2.6</v>
       </c>
       <c r="C93" t="n">
-        <v>2.9678</v>
+        <v>4</v>
       </c>
       <c r="D93" t="n">
-        <v>0.6445</v>
+        <v>1.2</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2191,10 +2191,10 @@
         <v>2.3</v>
       </c>
       <c r="C94" t="n">
-        <v>2.0928</v>
+        <v>3.3</v>
       </c>
       <c r="D94" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2210,10 +2210,10 @@
         <v>2.7</v>
       </c>
       <c r="C95" t="n">
-        <v>3.2178</v>
+        <v>4.2</v>
       </c>
       <c r="D95" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2229,10 +2229,10 @@
         <v>3</v>
       </c>
       <c r="C96" t="n">
-        <v>3.2178</v>
+        <v>4.2</v>
       </c>
       <c r="D96" t="n">
-        <v>0.6445</v>
+        <v>1.2</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>2.9</v>
       </c>
       <c r="C97" t="n">
-        <v>3.2178</v>
+        <v>4.2</v>
       </c>
       <c r="D97" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2267,10 +2267,10 @@
         <v>2.9</v>
       </c>
       <c r="C98" t="n">
-        <v>3.3428</v>
+        <v>4.3</v>
       </c>
       <c r="D98" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2286,10 +2286,10 @@
         <v>2.5</v>
       </c>
       <c r="C99" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D99" t="n">
-        <v>0.5195</v>
+        <v>1.1</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2305,10 +2305,10 @@
         <v>2.8</v>
       </c>
       <c r="C100" t="n">
-        <v>3.0928</v>
+        <v>4.1</v>
       </c>
       <c r="D100" t="n">
-        <v>0.7695</v>
+        <v>1.3</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2324,10 +2324,10 @@
         <v>3.3</v>
       </c>
       <c r="C101" t="n">
-        <v>7.0792</v>
+        <v>6</v>
       </c>
       <c r="D101" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2343,10 +2343,10 @@
         <v>2.7</v>
       </c>
       <c r="C102" t="n">
-        <v>5.9542</v>
+        <v>5.1</v>
       </c>
       <c r="D102" t="n">
-        <v>2.3925</v>
+        <v>1.9</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2362,10 +2362,10 @@
         <v>3</v>
       </c>
       <c r="C103" t="n">
-        <v>6.9542</v>
+        <v>5.9</v>
       </c>
       <c r="D103" t="n">
-        <v>2.6425</v>
+        <v>2.1</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2381,10 +2381,10 @@
         <v>2.9</v>
       </c>
       <c r="C104" t="n">
-        <v>6.5792</v>
+        <v>5.6</v>
       </c>
       <c r="D104" t="n">
-        <v>2.2675</v>
+        <v>1.8</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2400,10 +2400,10 @@
         <v>3</v>
       </c>
       <c r="C105" t="n">
-        <v>6.8292</v>
+        <v>5.8</v>
       </c>
       <c r="D105" t="n">
-        <v>2.7675</v>
+        <v>2.2</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2419,10 +2419,10 @@
         <v>3</v>
       </c>
       <c r="C106" t="n">
-        <v>7.5</v>
+        <v>6.6</v>
       </c>
       <c r="D106" t="n">
-        <v>2.6425</v>
+        <v>2.1</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2438,10 +2438,10 @@
         <v>2.5</v>
       </c>
       <c r="C107" t="n">
-        <v>5.2042</v>
+        <v>4.8756</v>
       </c>
       <c r="D107" t="n">
-        <v>2.1425</v>
+        <v>1.9035</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -2457,10 +2457,10 @@
         <v>2.9</v>
       </c>
       <c r="C108" t="n">
-        <v>7.4542</v>
+        <v>6.3</v>
       </c>
       <c r="D108" t="n">
-        <v>2.2675</v>
+        <v>1.8</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -2476,10 +2476,10 @@
         <v>2.5</v>
       </c>
       <c r="C109" t="n">
-        <v>6.8292</v>
+        <v>5.8</v>
       </c>
       <c r="D109" t="n">
-        <v>2.2675</v>
+        <v>1.8</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -2495,10 +2495,10 @@
         <v>3.6</v>
       </c>
       <c r="C110" t="n">
-        <v>7.2042</v>
+        <v>6.1</v>
       </c>
       <c r="D110" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -2514,10 +2514,10 @@
         <v>3.2</v>
       </c>
       <c r="C111" t="n">
-        <v>5.9542</v>
+        <v>5.1</v>
       </c>
       <c r="D111" t="n">
-        <v>2.5175</v>
+        <v>2</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -2533,10 +2533,10 @@
         <v>2.7</v>
       </c>
       <c r="C112" t="n">
-        <v>6.2042</v>
+        <v>5.3</v>
       </c>
       <c r="D112" t="n">
-        <v>2.3925</v>
+        <v>1.9</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -2552,10 +2552,10 @@
         <v>3</v>
       </c>
       <c r="C113" t="n">
-        <v>6.4542</v>
+        <v>5.5</v>
       </c>
       <c r="D113" t="n">
-        <v>2.6425</v>
+        <v>2.1</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -2571,10 +2571,10 @@
         <v>2.5</v>
       </c>
       <c r="C114" t="n">
-        <v>5.8292</v>
+        <v>5</v>
       </c>
       <c r="D114" t="n">
-        <v>2.5175</v>
+        <v>2</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -2590,10 +2590,10 @@
         <v>2.8</v>
       </c>
       <c r="C115" t="n">
-        <v>5.9542</v>
+        <v>5.1</v>
       </c>
       <c r="D115" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -2609,10 +2609,10 @@
         <v>3.2</v>
       </c>
       <c r="C116" t="n">
-        <v>6.2042</v>
+        <v>5.3</v>
       </c>
       <c r="D116" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -2628,10 +2628,10 @@
         <v>3</v>
       </c>
       <c r="C117" t="n">
-        <v>6.4542</v>
+        <v>5.5</v>
       </c>
       <c r="D117" t="n">
-        <v>2.2675</v>
+        <v>1.8</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -2647,10 +2647,10 @@
         <v>3.8</v>
       </c>
       <c r="C118" t="n">
-        <v>7.5</v>
+        <v>6.7</v>
       </c>
       <c r="D118" t="n">
-        <v>2.7675</v>
+        <v>2.2</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -2666,10 +2666,10 @@
         <v>2.6</v>
       </c>
       <c r="C119" t="n">
-        <v>7.5</v>
+        <v>6.9</v>
       </c>
       <c r="D119" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -2685,10 +2685,10 @@
         <v>2.2</v>
       </c>
       <c r="C120" t="n">
-        <v>5.8292</v>
+        <v>5.0729</v>
       </c>
       <c r="D120" t="n">
-        <v>1.8925</v>
+        <v>1.5395</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -2704,10 +2704,10 @@
         <v>3.2</v>
       </c>
       <c r="C121" t="n">
-        <v>6.7042</v>
+        <v>5.7</v>
       </c>
       <c r="D121" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -2723,10 +2723,10 @@
         <v>2.8</v>
       </c>
       <c r="C122" t="n">
-        <v>5.7042</v>
+        <v>4.9</v>
       </c>
       <c r="D122" t="n">
-        <v>2.5175</v>
+        <v>2</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -2742,10 +2742,10 @@
         <v>2.8</v>
       </c>
       <c r="C123" t="n">
-        <v>7.5</v>
+        <v>6.7</v>
       </c>
       <c r="D123" t="n">
-        <v>2.5175</v>
+        <v>2</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -2761,10 +2761,10 @@
         <v>2.7</v>
       </c>
       <c r="C124" t="n">
-        <v>5.7042</v>
+        <v>4.9245</v>
       </c>
       <c r="D124" t="n">
-        <v>2.2675</v>
+        <v>1.8133</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -2780,10 +2780,10 @@
         <v>3.3</v>
       </c>
       <c r="C125" t="n">
-        <v>6.7042</v>
+        <v>5.7</v>
       </c>
       <c r="D125" t="n">
-        <v>2.6425</v>
+        <v>2.1</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -2799,10 +2799,10 @@
         <v>3.2</v>
       </c>
       <c r="C126" t="n">
-        <v>7.0792</v>
+        <v>6</v>
       </c>
       <c r="D126" t="n">
-        <v>2.2675</v>
+        <v>1.8</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -2818,10 +2818,10 @@
         <v>2.8</v>
       </c>
       <c r="C127" t="n">
-        <v>5.5792</v>
+        <v>4.9018</v>
       </c>
       <c r="D127" t="n">
-        <v>2.2675</v>
+        <v>1.8552</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -2837,10 +2837,10 @@
         <v>3</v>
       </c>
       <c r="C128" t="n">
-        <v>5.7042</v>
+        <v>4.9245</v>
       </c>
       <c r="D128" t="n">
-        <v>2.2675</v>
+        <v>1.8133</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -2856,10 +2856,10 @@
         <v>2.8</v>
       </c>
       <c r="C129" t="n">
-        <v>6.5792</v>
+        <v>5.6</v>
       </c>
       <c r="D129" t="n">
-        <v>2.6425</v>
+        <v>2.1</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -2875,10 +2875,10 @@
         <v>3</v>
       </c>
       <c r="C130" t="n">
-        <v>6.8292</v>
+        <v>5.8</v>
       </c>
       <c r="D130" t="n">
-        <v>2.0175</v>
+        <v>1.6</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -2894,10 +2894,10 @@
         <v>2.8</v>
       </c>
       <c r="C131" t="n">
-        <v>7.2042</v>
+        <v>6.1</v>
       </c>
       <c r="D131" t="n">
-        <v>2.3925</v>
+        <v>1.9</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -2913,10 +2913,10 @@
         <v>3.8</v>
       </c>
       <c r="C132" t="n">
-        <v>7.5</v>
+        <v>6.4</v>
       </c>
       <c r="D132" t="n">
-        <v>2.5175</v>
+        <v>2</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -2932,10 +2932,10 @@
         <v>2.8</v>
       </c>
       <c r="C133" t="n">
-        <v>6.5792</v>
+        <v>5.6</v>
       </c>
       <c r="D133" t="n">
-        <v>2.7675</v>
+        <v>2.2</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -2951,10 +2951,10 @@
         <v>2.8</v>
       </c>
       <c r="C134" t="n">
-        <v>5.9542</v>
+        <v>5.1</v>
       </c>
       <c r="D134" t="n">
-        <v>1.8925</v>
+        <v>1.5</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -2970,10 +2970,10 @@
         <v>2.6</v>
       </c>
       <c r="C135" t="n">
-        <v>6.5792</v>
+        <v>5.6</v>
       </c>
       <c r="D135" t="n">
-        <v>1.7675</v>
+        <v>1.4</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -2989,10 +2989,10 @@
         <v>3</v>
       </c>
       <c r="C136" t="n">
-        <v>7.2042</v>
+        <v>6.1</v>
       </c>
       <c r="D136" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3008,10 +3008,10 @@
         <v>3.4</v>
       </c>
       <c r="C137" t="n">
-        <v>6.5792</v>
+        <v>5.6</v>
       </c>
       <c r="D137" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3027,10 +3027,10 @@
         <v>3.1</v>
       </c>
       <c r="C138" t="n">
-        <v>6.4542</v>
+        <v>5.5</v>
       </c>
       <c r="D138" t="n">
-        <v>2.2675</v>
+        <v>1.8</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3046,10 +3046,10 @@
         <v>3</v>
       </c>
       <c r="C139" t="n">
-        <v>5.5792</v>
+        <v>4.9018</v>
       </c>
       <c r="D139" t="n">
-        <v>2.2675</v>
+        <v>1.8552</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3065,10 +3065,10 @@
         <v>3.1</v>
       </c>
       <c r="C140" t="n">
-        <v>6.3292</v>
+        <v>5.4</v>
       </c>
       <c r="D140" t="n">
-        <v>2.6425</v>
+        <v>2.1</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3084,10 +3084,10 @@
         <v>3.1</v>
       </c>
       <c r="C141" t="n">
-        <v>6.5792</v>
+        <v>5.6</v>
       </c>
       <c r="D141" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3103,10 +3103,10 @@
         <v>3.1</v>
       </c>
       <c r="C142" t="n">
-        <v>5.9542</v>
+        <v>5.1</v>
       </c>
       <c r="D142" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3122,10 +3122,10 @@
         <v>2.7</v>
       </c>
       <c r="C143" t="n">
-        <v>5.9542</v>
+        <v>5.1</v>
       </c>
       <c r="D143" t="n">
-        <v>2.3925</v>
+        <v>1.9</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3141,10 +3141,10 @@
         <v>3.2</v>
       </c>
       <c r="C144" t="n">
-        <v>6.9542</v>
+        <v>5.9</v>
       </c>
       <c r="D144" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3160,10 +3160,10 @@
         <v>3.3</v>
       </c>
       <c r="C145" t="n">
-        <v>6.7042</v>
+        <v>5.7</v>
       </c>
       <c r="D145" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3179,10 +3179,10 @@
         <v>3</v>
       </c>
       <c r="C146" t="n">
-        <v>6.0792</v>
+        <v>5.2</v>
       </c>
       <c r="D146" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3198,10 +3198,10 @@
         <v>2.5</v>
       </c>
       <c r="C147" t="n">
-        <v>5.8292</v>
+        <v>5</v>
       </c>
       <c r="D147" t="n">
-        <v>2.3925</v>
+        <v>1.9</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -3217,10 +3217,10 @@
         <v>3</v>
       </c>
       <c r="C148" t="n">
-        <v>6.0792</v>
+        <v>5.2</v>
       </c>
       <c r="D148" t="n">
-        <v>2.5175</v>
+        <v>2</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -3236,10 +3236,10 @@
         <v>3.4</v>
       </c>
       <c r="C149" t="n">
-        <v>6.3292</v>
+        <v>5.4</v>
       </c>
       <c r="D149" t="n">
-        <v>2.8925</v>
+        <v>2.3</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>3</v>
       </c>
       <c r="C150" t="n">
-        <v>5.9542</v>
+        <v>5.1</v>
       </c>
       <c r="D150" t="n">
-        <v>2.2675</v>
+        <v>1.8</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>

</xml_diff>